<commit_message>
Added excel Data Input reading to rest
</commit_message>
<xml_diff>
--- a/java program/src/main/resources/testData.xlsx
+++ b/java program/src/main/resources/testData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" firstSheet="1" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" firstSheet="5" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="loginDataInputs" sheetId="1" r:id="rId1"/>
@@ -12,6 +12,10 @@
     <sheet name="BreadCrumbDataInput" sheetId="3" r:id="rId3"/>
     <sheet name="CurrencyDataInput" sheetId="4" r:id="rId4"/>
     <sheet name="ShoppingDataInput" sheetId="5" r:id="rId5"/>
+    <sheet name="SortDataInputs" sheetId="6" r:id="rId6"/>
+    <sheet name="SearchDataInputs" sheetId="7" r:id="rId7"/>
+    <sheet name="SearchCategoryDataInputs" sheetId="8" r:id="rId8"/>
+    <sheet name="CheckoutDataInput" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -23,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="63">
   <si>
     <t>Username</t>
   </si>
@@ -128,6 +132,90 @@
   </si>
   <si>
     <t>HP LP3065</t>
+  </si>
+  <si>
+    <t>Phones &amp; PDAs</t>
+  </si>
+  <si>
+    <t>Sort Tab</t>
+  </si>
+  <si>
+    <t>Cameras</t>
+  </si>
+  <si>
+    <t>Sorting A</t>
+  </si>
+  <si>
+    <t>Sorting B</t>
+  </si>
+  <si>
+    <t>Name (A - Z)</t>
+  </si>
+  <si>
+    <t>Name (Z - A)</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Mac</t>
+  </si>
+  <si>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>Components</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Keyword</t>
+  </si>
+  <si>
+    <t>Apple Cinema 30</t>
+  </si>
+  <si>
+    <t>Product Url</t>
+  </si>
+  <si>
+    <t>Product Name</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>Post</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>user</t>
+  </si>
+  <si>
+    <t>123 Test Street</t>
+  </si>
+  <si>
+    <t>Cairo</t>
+  </si>
+  <si>
+    <t>Egypt</t>
+  </si>
+  <si>
+    <t>Asyut</t>
   </si>
 </sst>
 </file>
@@ -172,7 +260,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -181,6 +269,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -682,7 +771,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B2" t="s">
@@ -693,9 +782,229 @@
       </c>
       <c r="D2" t="s">
         <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="21.6640625" customWidth="1"/>
+    <col min="3" max="3" width="26.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27.109375" customWidth="1"/>
+    <col min="2" max="2" width="24.6640625" customWidth="1"/>
+    <col min="3" max="3" width="22.44140625" customWidth="1"/>
+    <col min="4" max="4" width="30.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.21875" customWidth="1"/>
+    <col min="2" max="2" width="35.33203125" customWidth="1"/>
+    <col min="3" max="3" width="23.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="80.77734375" customWidth="1"/>
+    <col min="2" max="2" width="34.77734375" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" customWidth="1"/>
+    <col min="5" max="5" width="30.88671875" customWidth="1"/>
+    <col min="6" max="6" width="17.21875" customWidth="1"/>
+    <col min="7" max="7" width="18.5546875" customWidth="1"/>
+    <col min="8" max="8" width="21.5546875" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" customWidth="1"/>
+    <col min="10" max="10" width="14.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="4">
+        <v>45991</v>
+      </c>
+      <c r="D2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F2" t="s">
+        <v>59</v>
+      </c>
+      <c r="G2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H2">
+        <v>12345</v>
+      </c>
+      <c r="I2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>